<commit_message>
First fixes to handle negatives in splitting
Remove V>0,Y>0 constraints for MRIOT. For SUT, which asks for Y0 prior, allow to have negatives in Y0.
</commit_message>
<xml_diff>
--- a/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
+++ b/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4cb83e15a8550b8f/Documenti/GitHub/MARIO/mario/ops/cvxlab_models/Split_sectors/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\camic\Documents\GitHub\MARIO\mario\ops\cvxlab_models\Split_sectors\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="11_79969FA3E80A376F0FB1566667EC3185CD3110F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A0D34B11-099B-4BE6-B3B7-7D7EB8D6933E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59022F57-28C0-4712-841B-47F8FA912C4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="13185" yWindow="-16335" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="problem" sheetId="1" r:id="rId1"/>
@@ -583,7 +583,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -949,12 +949,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="3" max="3" width="100.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -968,12 +968,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4">
       <c r="B2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4">
       <c r="C3" t="s">
         <v>5</v>
       </c>
@@ -981,7 +981,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4">
       <c r="C4" t="s">
         <v>7</v>
       </c>
@@ -989,7 +989,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4">
       <c r="C5" t="s">
         <v>9</v>
       </c>
@@ -997,7 +997,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4">
       <c r="C6" t="s">
         <v>11</v>
       </c>
@@ -1005,7 +1005,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4">
       <c r="C7" t="s">
         <v>13</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4">
       <c r="C8" t="s">
         <v>15</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4">
       <c r="C9" t="s">
         <v>17</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4">
       <c r="C10" t="s">
         <v>19</v>
       </c>
@@ -1037,7 +1037,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4">
       <c r="C11" t="s">
         <v>21</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4">
       <c r="C12" t="s">
         <v>23</v>
       </c>
@@ -1053,7 +1053,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4">
       <c r="C13" t="s">
         <v>25</v>
       </c>
@@ -1061,7 +1061,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4">
       <c r="C14" t="s">
         <v>27</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4">
       <c r="C15" t="s">
         <v>29</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4">
       <c r="C16" t="s">
         <v>31</v>
       </c>
@@ -1085,7 +1085,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="3:4">
       <c r="C17" t="s">
         <v>33</v>
       </c>
@@ -1093,7 +1093,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="3:4">
       <c r="C18" t="s">
         <v>35</v>
       </c>
@@ -1101,7 +1101,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="3:4">
       <c r="C19" t="s">
         <v>37</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="3:4">
       <c r="C20" t="s">
         <v>39</v>
       </c>
@@ -1117,7 +1117,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="3:4">
       <c r="C21" t="s">
         <v>41</v>
       </c>
@@ -1125,7 +1125,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="3:4">
       <c r="C22" t="s">
         <v>43</v>
       </c>
@@ -1133,7 +1133,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="3:4">
       <c r="C23" t="s">
         <v>45</v>
       </c>
@@ -1149,9 +1149,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5">
       <c r="A1" s="1" t="s">
         <v>47</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5">
       <c r="A2" t="s">
         <v>51</v>
       </c>
@@ -1179,7 +1179,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5">
       <c r="A3" t="s">
         <v>54</v>
       </c>
@@ -1190,7 +1190,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -1198,7 +1198,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>58</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>60</v>
       </c>
@@ -1214,7 +1214,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5">
       <c r="A7" t="s">
         <v>62</v>
       </c>
@@ -1222,7 +1222,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5">
       <c r="A8" t="s">
         <v>64</v>
       </c>
@@ -1241,7 +1241,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Q51"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="12.81640625" customWidth="1"/>
     <col min="2" max="2" width="55.7265625" customWidth="1"/>
@@ -1256,7 +1256,7 @@
     <col min="12" max="12" width="11.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16">
       <c r="A1" s="1" t="s">
         <v>67</v>
       </c>
@@ -1306,7 +1306,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16">
       <c r="A2" t="s">
         <v>75</v>
       </c>
@@ -1335,7 +1335,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16">
       <c r="A3" t="s">
         <v>75</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16">
       <c r="A4" t="s">
         <v>75</v>
       </c>
@@ -1393,7 +1393,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16">
       <c r="A5" t="s">
         <v>88</v>
       </c>
@@ -1422,7 +1422,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16">
       <c r="A6" t="s">
         <v>92</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16">
       <c r="A7" t="s">
         <v>95</v>
       </c>
@@ -1474,7 +1474,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16">
       <c r="A8" t="s">
         <v>97</v>
       </c>
@@ -1500,7 +1500,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16">
       <c r="A9" t="s">
         <v>101</v>
       </c>
@@ -1529,7 +1529,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16">
       <c r="A10" t="s">
         <v>103</v>
       </c>
@@ -1558,7 +1558,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16">
       <c r="A11" t="s">
         <v>105</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16">
       <c r="A12" t="s">
         <v>106</v>
       </c>
@@ -1613,7 +1613,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16">
       <c r="A13" t="s">
         <v>107</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16">
       <c r="A14" t="s">
         <v>107</v>
       </c>
@@ -1671,7 +1671,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16">
       <c r="A15" t="s">
         <v>112</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16">
       <c r="A16" t="s">
         <v>112</v>
       </c>
@@ -1717,7 +1717,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15">
       <c r="A17" t="s">
         <v>116</v>
       </c>
@@ -1743,7 +1743,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15">
       <c r="A18" t="s">
         <v>116</v>
       </c>
@@ -1769,7 +1769,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15">
       <c r="A19" t="s">
         <v>122</v>
       </c>
@@ -1801,7 +1801,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15">
       <c r="A20" t="s">
         <v>122</v>
       </c>
@@ -1833,7 +1833,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15">
       <c r="A21" t="s">
         <v>122</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15">
       <c r="A22" t="s">
         <v>122</v>
       </c>
@@ -1897,7 +1897,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15">
       <c r="A23" t="s">
         <v>122</v>
       </c>
@@ -1929,7 +1929,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15">
       <c r="A24" t="s">
         <v>122</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15">
       <c r="A25" t="s">
         <v>122</v>
       </c>
@@ -1993,7 +1993,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15">
       <c r="A26" t="s">
         <v>131</v>
       </c>
@@ -2025,7 +2025,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15">
       <c r="A27" t="s">
         <v>131</v>
       </c>
@@ -2057,7 +2057,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15">
       <c r="A28" t="s">
         <v>131</v>
       </c>
@@ -2089,7 +2089,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15">
       <c r="A29" t="s">
         <v>136</v>
       </c>
@@ -2105,9 +2105,6 @@
       <c r="F29" t="s">
         <v>138</v>
       </c>
-      <c r="I29" t="b">
-        <v>1</v>
-      </c>
       <c r="J29" t="s">
         <v>104</v>
       </c>
@@ -2121,7 +2118,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15">
       <c r="A30" t="s">
         <v>136</v>
       </c>
@@ -2137,9 +2134,6 @@
       <c r="F30" t="s">
         <v>139</v>
       </c>
-      <c r="I30" t="b">
-        <v>1</v>
-      </c>
       <c r="J30" t="s">
         <v>104</v>
       </c>
@@ -2153,7 +2147,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15">
       <c r="A31" t="s">
         <v>136</v>
       </c>
@@ -2169,9 +2163,6 @@
       <c r="F31" t="s">
         <v>140</v>
       </c>
-      <c r="I31" t="b">
-        <v>1</v>
-      </c>
       <c r="J31" t="s">
         <v>100</v>
       </c>
@@ -2185,7 +2176,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15">
       <c r="A32" t="s">
         <v>141</v>
       </c>
@@ -2201,9 +2192,6 @@
       <c r="F32" t="s">
         <v>141</v>
       </c>
-      <c r="I32" t="b">
-        <v>1</v>
-      </c>
       <c r="K32" t="s">
         <v>121</v>
       </c>
@@ -2214,7 +2202,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:17">
       <c r="A33" t="s">
         <v>141</v>
       </c>
@@ -2230,9 +2218,6 @@
       <c r="F33" t="s">
         <v>142</v>
       </c>
-      <c r="I33" t="b">
-        <v>1</v>
-      </c>
       <c r="K33" t="s">
         <v>121</v>
       </c>
@@ -2243,7 +2228,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:17">
       <c r="A34" t="s">
         <v>143</v>
       </c>
@@ -2266,7 +2251,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:17">
       <c r="A35" t="s">
         <v>147</v>
       </c>
@@ -2298,7 +2283,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:17">
       <c r="A36" t="s">
         <v>150</v>
       </c>
@@ -2324,7 +2309,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:17">
       <c r="A37" t="s">
         <v>172</v>
       </c>
@@ -2356,7 +2341,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:17">
       <c r="A38" t="s">
         <v>152</v>
       </c>
@@ -2382,7 +2367,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:17">
       <c r="A39" t="s">
         <v>155</v>
       </c>
@@ -2405,7 +2390,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:17">
       <c r="A40" t="s">
         <v>157</v>
       </c>
@@ -2431,7 +2416,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:17">
       <c r="A41" t="s">
         <v>159</v>
       </c>
@@ -2457,7 +2442,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:17">
       <c r="A42" t="s">
         <v>161</v>
       </c>
@@ -2483,7 +2468,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:17">
       <c r="A43" t="s">
         <v>164</v>
       </c>
@@ -2512,7 +2497,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:17">
       <c r="A44" t="s">
         <v>168</v>
       </c>
@@ -2541,7 +2526,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:17">
       <c r="A45" t="s">
         <v>169</v>
       </c>
@@ -2570,7 +2555,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:17">
       <c r="A46" s="2" t="s">
         <v>173</v>
       </c>
@@ -2605,7 +2590,7 @@
       <c r="P46" s="2"/>
       <c r="Q46" s="2"/>
     </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:17">
       <c r="A47" s="2" t="s">
         <v>176</v>
       </c>
@@ -2638,7 +2623,7 @@
       <c r="P47" s="2"/>
       <c r="Q47" s="2"/>
     </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:17">
       <c r="A48" s="2" t="s">
         <v>179</v>
       </c>
@@ -2669,7 +2654,7 @@
       </c>
       <c r="Q48" s="2"/>
     </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:17">
       <c r="A49" s="2" t="s">
         <v>179</v>
       </c>
@@ -2700,7 +2685,7 @@
       </c>
       <c r="Q49" s="2"/>
     </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:17">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -2719,7 +2704,7 @@
       <c r="P50" s="2"/>
       <c r="Q50" s="2"/>
     </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:17">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -2744,14 +2729,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2950,21 +2933,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="90e7079a-7589-470d-892b-836f3f5ab9a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="9ef6bf99-292f-445d-95df-6a8984d5eb85" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82FFAD35-1A25-435C-B0F6-96A1B7601AC9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F46AB929-9659-4052-AEEC-F7A53C94BE55}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
-    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2989,9 +2971,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F46AB929-9659-4052-AEEC-F7A53C94BE55}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82FFAD35-1A25-435C-B0F6-96A1B7601AC9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="90e7079a-7589-470d-892b-836f3f5ab9a4"/>
+    <ds:schemaRef ds:uri="9ef6bf99-292f-445d-95df-6a8984d5eb85"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Fix for negative cells: now allowed in entropy minimization
Also fixed the cvxlab_bridge that was setting to zero all negative values when passing from database.db to MARIO format.
</commit_message>
<xml_diff>
--- a/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
+++ b/mario/ops/cvxlab_models/Split_sectors/model_settings.xlsx
@@ -36,7 +36,7 @@
     <t>description</t>
   </si>
   <si>
-    <t>Minimize(sum(entropy(Z_use_n,Z0_all_n))+sum(entropy(Z_use_st_p,Z0_st_p))+sum(entropy(V,V0)))</t>
+    <t>Minimize(sum(entropy(Z_use_n,Z0_all_n))+sum(entropy(Z_use_st_p,Z0_st_p))+sum(entropy_signed(V,V0)))</t>
   </si>
   <si>
     <t>Zold_p_st &lt;= (block_diag(I_p_pn,regions) @ Z_supply_to)*(1+eps)</t>
@@ -51,13 +51,13 @@
     <t>Constraint 1a(Z)-:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
   </si>
   <si>
-    <t>Yold &lt;= (block_diag(I_p_pn,regions) @ Y_pn_to)*(1+eps)</t>
+    <t>Yold-absval(Yold)*eps&lt;=(block_diag(I_p_pn,regions) @ Y_pn_to)</t>
   </si>
   <si>
     <t>Constraint 1a(Y)+:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
   </si>
   <si>
-    <t>Yold &gt;= (block_diag(I_p_pn,regions) @ Y_pn_to)*(1-eps)</t>
+    <t>Yold+absval(Yold)*eps&gt;=(block_diag(I_p_pn,regions) @ Y_pn_to)</t>
   </si>
   <si>
     <t>Constraint 1a(Y)-:  total consumption consistency by region and sector (excl. parent/) before and after the  sector addition</t>
@@ -87,13 +87,13 @@
     <t>Constraint 1c-:  total consumption consistency by region and sector (parent/ use of stables) before and after the  sector addition</t>
   </si>
   <si>
-    <t>Vold &lt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1+eps)</t>
+    <t>Vold-absval(Vold)*eps&lt;=(V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))</t>
   </si>
   <si>
     <t>Constraint 1d+: VA consistency</t>
   </si>
   <si>
-    <t>Vold &gt;= (V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))*(1-eps)</t>
+    <t>Vold+absval(Vold)*eps&gt;=(V @ tran(block_diag(I_p_pn,regions) ) @ tran(I_p_r_from_to))</t>
   </si>
   <si>
     <t>Constraint 1d-: VA consistency</t>

</xml_diff>